<commit_message>
Update slr_evidence.xlsx with revised content
</commit_message>
<xml_diff>
--- a/slr_evidence.xlsx
+++ b/slr_evidence.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tartu\4th Semester\Masters Thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7660D65-90A7-4577-8505-9ACAAB4DA795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6C64B9-5437-4389-817A-8A5B8DE29633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -474,10 +474,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -787,14 +796,14 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.36328125" customWidth="1"/>
-    <col min="3" max="3" width="59.1796875" customWidth="1"/>
-    <col min="4" max="4" width="21.54296875" customWidth="1"/>
-    <col min="5" max="5" width="29.81640625" customWidth="1"/>
-    <col min="6" max="6" width="26.90625" customWidth="1"/>
-    <col min="7" max="7" width="23.54296875" customWidth="1"/>
+    <col min="3" max="3" width="39.453125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="18.81640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="26.90625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="23.54296875" style="4" customWidth="1"/>
     <col min="8" max="8" width="16.6328125" customWidth="1"/>
-    <col min="9" max="9" width="17.90625" customWidth="1"/>
-    <col min="10" max="10" width="44.7265625" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="29.453125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -804,782 +813,860 @@
       <c r="B1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2">
+    <row r="2" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" s="2">
+        <v>26</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="4" t="s">
         <v>76</v>
       </c>
       <c r="H2" t="s">
         <v>128</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="4" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="3" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B3" s="2">
+        <v>31</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="4" t="s">
         <v>77</v>
       </c>
       <c r="H3" t="s">
         <v>96</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="4" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="4" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B4" s="2">
+        <v>37</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="4" t="s">
         <v>78</v>
       </c>
       <c r="H4" t="s">
         <v>98</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="4" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B5" s="2">
+        <v>38</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="4" t="s">
         <v>79</v>
       </c>
       <c r="H5" t="s">
         <v>98</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="4" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B6" s="2">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="4" t="s">
         <v>80</v>
       </c>
       <c r="H6" t="s">
         <v>128</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="4" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="7" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B7" s="2">
+        <v>39</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="4" t="s">
         <v>81</v>
       </c>
       <c r="H7" t="s">
         <v>96</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B8" s="2">
+        <v>40</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="4" t="s">
         <v>82</v>
       </c>
       <c r="H8" t="s">
         <v>96</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="4" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9">
+    <row r="9" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="C9" t="s">
+      <c r="B9" s="2">
+        <v>20</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="4" t="s">
         <v>83</v>
       </c>
       <c r="H9" t="s">
         <v>94</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="4" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10">
+    <row r="10" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="C10" t="s">
+      <c r="B10" s="2">
+        <v>41</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="4" t="s">
         <v>84</v>
       </c>
       <c r="H10" t="s">
         <v>98</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="4" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="C11" t="s">
+      <c r="B11" s="2">
+        <v>27</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="4" t="s">
         <v>85</v>
       </c>
       <c r="H11" t="s">
         <v>96</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="4" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="C12" t="s">
+      <c r="B12" s="2">
+        <v>28</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="4" t="s">
         <v>86</v>
       </c>
       <c r="H12" t="s">
         <v>96</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="4" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13">
+    <row r="13" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="C13" t="s">
+      <c r="B13" s="2">
+        <v>36</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="4" t="s">
         <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>96</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="4" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="C14" t="s">
+      <c r="B14" s="2">
+        <v>33</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="4" t="s">
         <v>87</v>
       </c>
       <c r="H14" t="s">
         <v>128</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="4" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B15" s="2">
+        <v>34</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="4" t="s">
         <v>88</v>
       </c>
       <c r="H15" t="s">
         <v>96</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="4" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="C16" t="s">
+      <c r="B16" s="2">
+        <v>2</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="4" t="s">
         <v>89</v>
       </c>
       <c r="H16" t="s">
         <v>96</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="4" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="C17" t="s">
+      <c r="B17" s="2">
+        <v>42</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="4" t="s">
         <v>90</v>
       </c>
       <c r="H17" t="s">
         <v>96</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="4" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18">
+    <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="C18" t="s">
+      <c r="B18" s="2">
+        <v>43</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="4" t="s">
         <v>91</v>
       </c>
       <c r="H18" t="s">
         <v>98</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I18" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="4" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="C19" t="s">
+      <c r="B19" s="2">
+        <v>29</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="4" t="s">
         <v>92</v>
       </c>
       <c r="H19" t="s">
         <v>96</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="4" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20">
+    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="C20" t="s">
+      <c r="B20" s="2">
+        <v>44</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="4" t="s">
         <v>93</v>
       </c>
       <c r="H20" t="s">
         <v>98</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="4" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21">
+    <row r="21" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="C21" t="s">
+      <c r="B21" s="2">
+        <v>46</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="4" t="s">
         <v>94</v>
       </c>
       <c r="H21" t="s">
         <v>94</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="4" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22">
+    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
         <v>21</v>
       </c>
-      <c r="C22" t="s">
+      <c r="B22" s="2">
+        <v>47</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="4" t="s">
         <v>94</v>
       </c>
       <c r="H22" t="s">
         <v>94</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="4" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23">
+    <row r="23" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
         <v>22</v>
       </c>
-      <c r="C23" t="s">
+      <c r="B23" s="2">
+        <v>32</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="4" t="s">
         <v>95</v>
       </c>
       <c r="H23" t="s">
         <v>128</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="4" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24">
+      <c r="A24" s="2">
         <v>23</v>
       </c>
-      <c r="C24" t="s">
+      <c r="B24" s="2">
         <v>30</v>
       </c>
-      <c r="D24" t="s">
+      <c r="C24" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="4" t="s">
         <v>96</v>
       </c>
       <c r="H24" t="s">
         <v>96</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="4" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25">
+      <c r="A25" s="2">
         <v>24</v>
       </c>
-      <c r="C25" t="s">
+      <c r="B25" s="2">
+        <v>45</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="4" t="s">
         <v>97</v>
       </c>
       <c r="H25" t="s">
         <v>98</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="4" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26">
+    <row r="26" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
         <v>25</v>
       </c>
-      <c r="C26" t="s">
+      <c r="B26" s="2">
+        <v>35</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="4" t="s">
         <v>87</v>
       </c>
       <c r="H26" t="s">
         <v>128</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="4" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27">
+    <row r="27" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="C27" t="s">
+      <c r="B27" s="2">
+        <v>48</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="4" t="s">
         <v>94</v>
       </c>
       <c r="H27" t="s">
         <v>94</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="4" t="s">
         <v>125</v>
       </c>
     </row>

</xml_diff>